<commit_message>
add the customer enum and ACS, alarmHistory
</commit_message>
<xml_diff>
--- a/OutputResults/BSBU_AccountSettingPage_AdminPortal.xlsx
+++ b/OutputResults/BSBU_AccountSettingPage_AdminPortal.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2722" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2736" uniqueCount="79">
   <si>
     <t/>
   </si>
@@ -293,7 +293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W130"/>
+  <dimension ref="A1:W132"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -4585,6 +4585,28 @@
         <v>4661.0</v>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B131" t="n" s="0">
+        <v>1674.0</v>
+      </c>
+      <c r="C131" t="n" s="0">
+        <v>3893.0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B132" t="n" s="0">
+        <v>2301.0</v>
+      </c>
+      <c r="C132" t="n" s="0">
+        <v>5888.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>